<commit_message>
create backups of overridden entries to prevent full deletion
</commit_message>
<xml_diff>
--- a/uncategorized_suggestions.xlsx
+++ b/uncategorized_suggestions.xlsx
@@ -4133,9 +4133,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G71" s="15" t="inlineStr"/>
-      <c r="H71" s="15" t="inlineStr"/>
-      <c r="I71" s="15" t="inlineStr"/>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I71" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J71" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 4; Politico-Military Issues: 3; Science and Technology: 1</t>
@@ -4169,9 +4181,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G72" s="15" t="inlineStr"/>
-      <c r="H72" s="15" t="inlineStr"/>
-      <c r="I72" s="15" t="inlineStr"/>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J72" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 4; Warfare: 3; Bilateral Relations: 1</t>
@@ -4205,9 +4229,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G73" s="15" t="inlineStr"/>
-      <c r="H73" s="15" t="inlineStr"/>
-      <c r="I73" s="15" t="inlineStr"/>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I73" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J73" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 4; Global Issues: 2; Science and Technology: 1</t>
@@ -4241,9 +4277,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G74" s="15" t="inlineStr"/>
-      <c r="H74" s="15" t="inlineStr"/>
-      <c r="I74" s="15" t="inlineStr"/>
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J74" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 45; Foreign Economic Policy: 15; Arms Control and Disarmament: 13</t>
@@ -4277,9 +4325,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G75" s="15" t="inlineStr"/>
-      <c r="H75" s="15" t="inlineStr"/>
-      <c r="I75" s="15" t="inlineStr"/>
+      <c r="G75" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H75" s="15" t="inlineStr">
+        <is>
+          <t>Energy and Natural Resources</t>
+        </is>
+      </c>
+      <c r="I75" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J75" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 42; Politico-Military Issues: 13; Global Issues: 12</t>
@@ -4313,9 +4373,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G76" s="15" t="inlineStr"/>
-      <c r="H76" s="15" t="inlineStr"/>
-      <c r="I76" s="15" t="inlineStr"/>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J76" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 27; Global Issues: 8; Foreign Economic Policy: 7</t>
@@ -4349,9 +4421,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G77" s="15" t="inlineStr"/>
-      <c r="H77" s="15" t="inlineStr"/>
-      <c r="I77" s="15" t="inlineStr"/>
+      <c r="G77" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Nonproliferation</t>
+        </is>
+      </c>
+      <c r="I77" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J77" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 7; Global Issues: 1; Politico-Military Issues: 1</t>
@@ -4385,9 +4469,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G78" s="15" t="inlineStr"/>
-      <c r="H78" s="15" t="inlineStr"/>
-      <c r="I78" s="15" t="inlineStr"/>
+      <c r="G78" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I78" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J78" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 29; Global Issues: 8; Information Programs: 4</t>
@@ -4421,9 +4517,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G79" s="15" t="inlineStr"/>
-      <c r="H79" s="15" t="inlineStr"/>
-      <c r="I79" s="15" t="inlineStr"/>
+      <c r="G79" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I79" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J79" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 405; Politico-Military Issues: 178; Foreign Economic Policy: 108</t>
@@ -4457,9 +4565,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G80" s="15" t="inlineStr"/>
-      <c r="H80" s="15" t="inlineStr"/>
-      <c r="I80" s="15" t="inlineStr"/>
+      <c r="G80" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H80" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I80" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J80" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 12; Department of State: 3; Global Issues: 3</t>
@@ -4493,9 +4613,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G81" s="15" t="inlineStr"/>
-      <c r="H81" s="15" t="inlineStr"/>
-      <c r="I81" s="15" t="inlineStr"/>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J81" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 104; Global Issues: 20; Politico-Military Issues: 18</t>
@@ -4529,9 +4661,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G82" s="15" t="inlineStr"/>
-      <c r="H82" s="15" t="inlineStr"/>
-      <c r="I82" s="15" t="inlineStr"/>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Aid</t>
+        </is>
+      </c>
+      <c r="I82" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J82" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 8; Politico-Military Issues: 2; Global Issues: 2</t>
@@ -4565,9 +4709,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G83" s="15" t="inlineStr"/>
-      <c r="H83" s="15" t="inlineStr"/>
-      <c r="I83" s="15" t="inlineStr"/>
+      <c r="G83" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H83" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I83" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J83" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 4; Politico-Military Issues: 2; Foreign Economic Policy: 1</t>
@@ -4601,9 +4757,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G84" s="15" t="inlineStr"/>
-      <c r="H84" s="15" t="inlineStr"/>
-      <c r="I84" s="15" t="inlineStr"/>
+      <c r="G84" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H84" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I84" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J84" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 66; Politico-Military Issues: 25; Global Issues: 15</t>
@@ -4637,9 +4805,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G85" s="15" t="inlineStr"/>
-      <c r="H85" s="15" t="inlineStr"/>
-      <c r="I85" s="15" t="inlineStr"/>
+      <c r="G85" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H85" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I85" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J85" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 5; Politico-Military Issues: 3; Global Issues: 2</t>
@@ -4673,9 +4853,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G86" s="15" t="inlineStr"/>
-      <c r="H86" s="15" t="inlineStr"/>
-      <c r="I86" s="15" t="inlineStr"/>
+      <c r="G86" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H86" s="15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="I86" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J86" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 187; Politico-Military Issues: 56; Human Rights: 55</t>
@@ -4709,9 +4901,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G87" s="15" t="inlineStr"/>
-      <c r="H87" s="15" t="inlineStr"/>
-      <c r="I87" s="15" t="inlineStr"/>
+      <c r="G87" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H87" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I87" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J87" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 47; Global Issues: 14; Arms Control and Disarmament: 7</t>
@@ -4745,9 +4949,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G88" s="15" t="inlineStr"/>
-      <c r="H88" s="15" t="inlineStr"/>
-      <c r="I88" s="15" t="inlineStr"/>
+      <c r="G88" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H88" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I88" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J88" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 6; Global Issues: 3; Bilateral Relations: 2</t>
@@ -4781,9 +4997,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G89" s="15" t="inlineStr"/>
-      <c r="H89" s="15" t="inlineStr"/>
-      <c r="I89" s="15" t="inlineStr"/>
+      <c r="G89" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H89" s="15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="I89" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J89" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 2; Human Rights: 2; Politico-Military Issues: 1</t>
@@ -4817,9 +5045,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G90" s="15" t="inlineStr"/>
-      <c r="H90" s="15" t="inlineStr"/>
-      <c r="I90" s="15" t="inlineStr"/>
+      <c r="G90" s="15" t="inlineStr">
+        <is>
+          <t>Information Programs</t>
+        </is>
+      </c>
+      <c r="H90" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I90" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J90" s="18" t="inlineStr">
         <is>
           <t>Information Programs: 4; Bilateral Relations: 2; Politico-Military Issues: 1</t>
@@ -4853,9 +5093,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G91" s="15" t="inlineStr"/>
-      <c r="H91" s="15" t="inlineStr"/>
-      <c r="I91" s="15" t="inlineStr"/>
+      <c r="G91" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H91" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I91" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J91" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 1297; Politico-Military Issues: 324; Global Issues: 159</t>
@@ -4889,9 +5141,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G92" s="15" t="inlineStr"/>
-      <c r="H92" s="15" t="inlineStr"/>
-      <c r="I92" s="15" t="inlineStr"/>
+      <c r="G92" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H92" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I92" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J92" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 238; Politico-Military Issues: 52; Global Issues: 29</t>
@@ -4925,9 +5189,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G93" s="15" t="inlineStr"/>
-      <c r="H93" s="15" t="inlineStr"/>
-      <c r="I93" s="15" t="inlineStr"/>
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H93" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I93" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J93" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 25; Global Issues: 4; Human Rights: 4</t>
@@ -4961,9 +5237,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G94" s="15" t="inlineStr"/>
-      <c r="H94" s="15" t="inlineStr"/>
-      <c r="I94" s="15" t="inlineStr"/>
+      <c r="G94" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H94" s="15" t="inlineStr">
+        <is>
+          <t>Refugees</t>
+        </is>
+      </c>
+      <c r="I94" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J94" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 7; Global Issues: 3; Department of State: 2</t>
@@ -4997,9 +5285,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G95" s="15" t="inlineStr"/>
-      <c r="H95" s="15" t="inlineStr"/>
-      <c r="I95" s="15" t="inlineStr"/>
+      <c r="G95" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I95" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J95" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 14; Arms Control and Disarmament: 6; Foreign Economic Policy: 3</t>
@@ -5033,9 +5333,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G96" s="15" t="inlineStr"/>
-      <c r="H96" s="15" t="inlineStr"/>
-      <c r="I96" s="15" t="inlineStr"/>
+      <c r="G96" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H96" s="15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="I96" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J96" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 95; Global Issues: 18; Human Rights: 17</t>
@@ -5069,9 +5381,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G97" s="15" t="inlineStr"/>
-      <c r="H97" s="15" t="inlineStr"/>
-      <c r="I97" s="15" t="inlineStr"/>
+      <c r="G97" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H97" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I97" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J97" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 25; Politico-Military Issues: 15; Science and Technology: 6</t>
@@ -5105,9 +5429,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G98" s="15" t="inlineStr"/>
-      <c r="H98" s="15" t="inlineStr"/>
-      <c r="I98" s="15" t="inlineStr"/>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H98" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I98" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J98" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 252; Politico-Military Issues: 93; Foreign Economic Policy: 36</t>
@@ -5141,9 +5477,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G99" s="15" t="inlineStr"/>
-      <c r="H99" s="15" t="inlineStr"/>
-      <c r="I99" s="15" t="inlineStr"/>
+      <c r="G99" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H99" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I99" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J99" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 1876; Politico-Military Issues: 383; Bilateral Relations: 332</t>
@@ -5177,9 +5525,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G100" s="15" t="inlineStr"/>
-      <c r="H100" s="15" t="inlineStr"/>
-      <c r="I100" s="15" t="inlineStr"/>
+      <c r="G100" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H100" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I100" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J100" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 30; Politico-Military Issues: 12; Bilateral Relations: 9</t>
@@ -5213,9 +5573,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G101" s="15" t="inlineStr"/>
-      <c r="H101" s="15" t="inlineStr"/>
-      <c r="I101" s="15" t="inlineStr"/>
+      <c r="G101" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H101" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I101" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J101" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 625; Politico-Military Issues: 155; Global Issues: 91</t>
@@ -5249,9 +5621,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G102" s="15" t="inlineStr"/>
-      <c r="H102" s="15" t="inlineStr"/>
-      <c r="I102" s="15" t="inlineStr"/>
+      <c r="G102" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H102" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I102" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J102" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 102; Politico-Military Issues: 34; International Law: 14</t>
@@ -5285,9 +5669,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G103" s="15" t="inlineStr"/>
-      <c r="H103" s="15" t="inlineStr"/>
-      <c r="I103" s="15" t="inlineStr"/>
+      <c r="G103" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H103" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I103" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J103" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 35; Politico-Military Issues: 8; Global Issues: 8</t>
@@ -5321,9 +5717,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G104" s="15" t="inlineStr"/>
-      <c r="H104" s="15" t="inlineStr"/>
-      <c r="I104" s="15" t="inlineStr"/>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H104" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I104" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J104" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 238; Politico-Military Issues: 72; International Law: 41</t>
@@ -5357,9 +5765,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G105" s="15" t="inlineStr"/>
-      <c r="H105" s="15" t="inlineStr"/>
-      <c r="I105" s="15" t="inlineStr"/>
+      <c r="G105" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H105" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I105" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J105" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 195; Politico-Military Issues: 85; Global Issues: 52</t>
@@ -5393,9 +5813,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G106" s="15" t="inlineStr"/>
-      <c r="H106" s="15" t="inlineStr"/>
-      <c r="I106" s="15" t="inlineStr"/>
+      <c r="G106" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H106" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I106" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J106" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 277; Politico-Military Issues: 84; International Law: 57</t>
@@ -5429,9 +5861,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G107" s="15" t="inlineStr"/>
-      <c r="H107" s="15" t="inlineStr"/>
-      <c r="I107" s="15" t="inlineStr"/>
+      <c r="G107" s="15" t="inlineStr">
+        <is>
+          <t>International Law</t>
+        </is>
+      </c>
+      <c r="H107" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I107" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J107" s="18" t="inlineStr">
         <is>
           <t>Global Issues: 1; Human Rights: 1</t>
@@ -5465,9 +5909,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G108" s="15" t="inlineStr"/>
-      <c r="H108" s="15" t="inlineStr"/>
-      <c r="I108" s="15" t="inlineStr"/>
+      <c r="G108" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H108" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I108" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J108" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 33; Global Issues: 11; Politico-Military Issues: 5</t>
@@ -5501,9 +5957,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G109" s="15" t="inlineStr"/>
-      <c r="H109" s="15" t="inlineStr"/>
-      <c r="I109" s="15" t="inlineStr"/>
+      <c r="G109" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H109" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J109" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 1; Arms Control and Disarmament: 1</t>
@@ -5537,9 +6005,21 @@
           <t>co-occurrence</t>
         </is>
       </c>
-      <c r="G110" s="15" t="inlineStr"/>
-      <c r="H110" s="15" t="inlineStr"/>
-      <c r="I110" s="15" t="inlineStr"/>
+      <c r="G110" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H110" s="15" t="inlineStr">
+        <is>
+          <t>Religious Freedom</t>
+        </is>
+      </c>
+      <c r="I110" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J110" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 7; Global Issues: 4; Foreign Economic Policy: 2</t>
@@ -5573,9 +6053,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G111" s="15" t="inlineStr"/>
-      <c r="H111" s="15" t="inlineStr"/>
-      <c r="I111" s="15" t="inlineStr"/>
+      <c r="G111" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H111" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I111" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J111" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 154; Arms Control and Disarmament: 84; Politico-Military Issues: 61</t>
@@ -5609,9 +6101,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G112" s="15" t="inlineStr"/>
-      <c r="H112" s="15" t="inlineStr"/>
-      <c r="I112" s="15" t="inlineStr"/>
+      <c r="G112" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H112" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I112" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J112" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 25; Global Issues: 8; Bilateral Relations: 7</t>
@@ -5645,9 +6149,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G113" s="15" t="inlineStr"/>
-      <c r="H113" s="15" t="inlineStr"/>
-      <c r="I113" s="15" t="inlineStr"/>
+      <c r="G113" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H113" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I113" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J113" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 45; Politico-Military Issues: 11; Global Issues: 8</t>
@@ -5681,9 +6197,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G114" s="15" t="inlineStr"/>
-      <c r="H114" s="15" t="inlineStr"/>
-      <c r="I114" s="15" t="inlineStr"/>
+      <c r="G114" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H114" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I114" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J114" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 48; Politico-Military Issues: 26; Global Issues: 20</t>
@@ -5717,9 +6245,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G115" s="15" t="inlineStr"/>
-      <c r="H115" s="15" t="inlineStr"/>
-      <c r="I115" s="15" t="inlineStr"/>
+      <c r="G115" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H115" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I115" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J115" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 17; International Law: 4; Department of State: 4</t>
@@ -5753,9 +6293,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G116" s="15" t="inlineStr"/>
-      <c r="H116" s="15" t="inlineStr"/>
-      <c r="I116" s="15" t="inlineStr"/>
+      <c r="G116" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H116" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I116" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J116" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 187; Politico-Military Issues: 49; Global Issues: 38</t>
@@ -5789,9 +6341,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G117" s="15" t="inlineStr"/>
-      <c r="H117" s="15" t="inlineStr"/>
-      <c r="I117" s="15" t="inlineStr"/>
+      <c r="G117" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H117" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I117" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J117" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 16; Foreign Economic Policy: 8; Human Rights: 6</t>
@@ -5825,9 +6389,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G118" s="15" t="inlineStr"/>
-      <c r="H118" s="15" t="inlineStr"/>
-      <c r="I118" s="15" t="inlineStr"/>
+      <c r="G118" s="15" t="inlineStr">
+        <is>
+          <t>Bilateral Relations</t>
+        </is>
+      </c>
+      <c r="H118" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I118" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J118" s="18" t="inlineStr">
         <is>
           <t>Bilateral Relations: 3; Information Programs: 1; Human Rights: 1</t>
@@ -5861,9 +6437,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G119" s="15" t="inlineStr"/>
-      <c r="H119" s="15" t="inlineStr"/>
-      <c r="I119" s="15" t="inlineStr"/>
+      <c r="G119" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H119" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I119" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J119" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 4; Warfare: 2; Science and Technology: 2</t>
@@ -5897,9 +6485,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G120" s="15" t="inlineStr"/>
-      <c r="H120" s="15" t="inlineStr"/>
-      <c r="I120" s="15" t="inlineStr"/>
+      <c r="G120" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H120" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I120" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J120" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 4; Politico-Military Issues: 3; Bilateral Relations: 2</t>
@@ -5933,9 +6533,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G121" s="15" t="inlineStr"/>
-      <c r="H121" s="15" t="inlineStr"/>
-      <c r="I121" s="15" t="inlineStr"/>
+      <c r="G121" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H121" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I121" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J121" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 53; Foreign Economic Policy: 27; Politico-Military Issues: 21</t>
@@ -5969,9 +6581,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G122" s="15" t="inlineStr"/>
-      <c r="H122" s="15" t="inlineStr"/>
-      <c r="I122" s="15" t="inlineStr"/>
+      <c r="G122" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H122" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I122" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J122" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 75; Human Rights: 20; Politico-Military Issues: 18</t>
@@ -6005,9 +6629,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G123" s="15" t="inlineStr"/>
-      <c r="H123" s="15" t="inlineStr"/>
-      <c r="I123" s="15" t="inlineStr"/>
+      <c r="G123" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H123" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I123" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J123" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 133; Politico-Military Issues: 41; Global Issues: 24</t>
@@ -6041,9 +6677,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G124" s="15" t="inlineStr"/>
-      <c r="H124" s="15" t="inlineStr"/>
-      <c r="I124" s="15" t="inlineStr"/>
+      <c r="G124" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H124" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I124" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J124" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 327; Politico-Military Issues: 211; Arms Control and Disarmament: 166</t>
@@ -6077,9 +6725,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G125" s="15" t="inlineStr"/>
-      <c r="H125" s="15" t="inlineStr"/>
-      <c r="I125" s="15" t="inlineStr"/>
+      <c r="G125" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H125" s="15" t="inlineStr">
+        <is>
+          <t>Immigration</t>
+        </is>
+      </c>
+      <c r="I125" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J125" s="18" t="inlineStr">
         <is>
           <t>Global Issues: 7; Human Rights: 5; Politico-Military Issues: 2</t>
@@ -6113,9 +6773,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G126" s="15" t="inlineStr"/>
-      <c r="H126" s="15" t="inlineStr"/>
-      <c r="I126" s="15" t="inlineStr"/>
+      <c r="G126" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H126" s="15" t="inlineStr">
+        <is>
+          <t>Energy and Natural Resources</t>
+        </is>
+      </c>
+      <c r="I126" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J126" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 6; Science and Technology: 2; Bilateral Relations: 2</t>
@@ -6149,9 +6821,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G127" s="15" t="inlineStr"/>
-      <c r="H127" s="15" t="inlineStr"/>
-      <c r="I127" s="15" t="inlineStr"/>
+      <c r="G127" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H127" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I127" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J127" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 236; Politico-Military Issues: 75; Arms Control and Disarmament: 52</t>
@@ -6185,9 +6869,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G128" s="15" t="inlineStr"/>
-      <c r="H128" s="15" t="inlineStr"/>
-      <c r="I128" s="15" t="inlineStr"/>
+      <c r="G128" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H128" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I128" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J128" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 46; Global Issues: 18; Politico-Military Issues: 9</t>
@@ -6221,9 +6917,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G129" s="15" t="inlineStr"/>
-      <c r="H129" s="15" t="inlineStr"/>
-      <c r="I129" s="15" t="inlineStr"/>
+      <c r="G129" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H129" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I129" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J129" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 623; Politico-Military Issues: 192; Global Issues: 123</t>
@@ -6257,9 +6965,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G130" s="15" t="inlineStr"/>
-      <c r="H130" s="15" t="inlineStr"/>
-      <c r="I130" s="15" t="inlineStr"/>
+      <c r="G130" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H130" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I130" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J130" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 25; Bilateral Relations: 8; Global Issues: 6</t>
@@ -6293,9 +7013,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G131" s="15" t="inlineStr"/>
-      <c r="H131" s="15" t="inlineStr"/>
-      <c r="I131" s="15" t="inlineStr"/>
+      <c r="G131" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H131" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I131" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J131" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 150; Politico-Military Issues: 71; Foreign Economic Policy: 44</t>
@@ -6329,9 +7061,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G132" s="15" t="inlineStr"/>
-      <c r="H132" s="15" t="inlineStr"/>
-      <c r="I132" s="15" t="inlineStr"/>
+      <c r="G132" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H132" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I132" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J132" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 212; Politico-Military Issues: 67; Global Issues: 65</t>
@@ -6365,9 +7109,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G133" s="15" t="inlineStr"/>
-      <c r="H133" s="15" t="inlineStr"/>
-      <c r="I133" s="15" t="inlineStr"/>
+      <c r="G133" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H133" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I133" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J133" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 18; International Law: 6; Politico-Military Issues: 5</t>
@@ -6401,9 +7157,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G134" s="15" t="inlineStr"/>
-      <c r="H134" s="15" t="inlineStr"/>
-      <c r="I134" s="15" t="inlineStr"/>
+      <c r="G134" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H134" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I134" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J134" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 6; Science and Technology: 3; Information Programs: 3</t>
@@ -6437,9 +7205,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G135" s="15" t="inlineStr"/>
-      <c r="H135" s="15" t="inlineStr"/>
-      <c r="I135" s="15" t="inlineStr"/>
+      <c r="G135" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H135" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I135" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J135" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 134; Politico-Military Issues: 40; Global Issues: 31</t>
@@ -6473,9 +7253,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G136" s="15" t="inlineStr"/>
-      <c r="H136" s="15" t="inlineStr"/>
-      <c r="I136" s="15" t="inlineStr"/>
+      <c r="G136" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H136" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I136" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J136" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 96; Global Issues: 25; Politico-Military Issues: 24</t>
@@ -6509,9 +7301,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G137" s="15" t="inlineStr"/>
-      <c r="H137" s="15" t="inlineStr"/>
-      <c r="I137" s="15" t="inlineStr"/>
+      <c r="G137" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H137" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I137" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J137" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 166; Politico-Military Issues: 51; Human Rights: 33</t>
@@ -6545,9 +7349,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G138" s="15" t="inlineStr"/>
-      <c r="H138" s="15" t="inlineStr"/>
-      <c r="I138" s="15" t="inlineStr"/>
+      <c r="G138" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H138" s="15" t="inlineStr">
+        <is>
+          <t>HIV/AIDS</t>
+        </is>
+      </c>
+      <c r="I138" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J138" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 4; Global Issues: 2; Department of State: 2</t>
@@ -6581,9 +7397,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G139" s="15" t="inlineStr"/>
-      <c r="H139" s="15" t="inlineStr"/>
-      <c r="I139" s="15" t="inlineStr"/>
+      <c r="G139" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H139" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I139" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J139" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 4; Global Issues: 2; Science and Technology: 1</t>
@@ -6617,9 +7445,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G140" s="15" t="inlineStr"/>
-      <c r="H140" s="15" t="inlineStr"/>
-      <c r="I140" s="15" t="inlineStr"/>
+      <c r="G140" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H140" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I140" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J140" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 73; Politico-Military Issues: 26; International Law: 15</t>
@@ -6653,9 +7493,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G141" s="15" t="inlineStr"/>
-      <c r="H141" s="15" t="inlineStr"/>
-      <c r="I141" s="15" t="inlineStr"/>
+      <c r="G141" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H141" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I141" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J141" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 773; Bilateral Relations: 217; Global Issues: 180</t>
@@ -6689,9 +7541,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G142" s="15" t="inlineStr"/>
-      <c r="H142" s="15" t="inlineStr"/>
-      <c r="I142" s="15" t="inlineStr"/>
+      <c r="G142" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H142" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I142" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J142" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 107; Foreign Economic Policy: 57; Arms Control and Disarmament: 45</t>
@@ -6725,9 +7589,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G143" s="15" t="inlineStr"/>
-      <c r="H143" s="15" t="inlineStr"/>
-      <c r="I143" s="15" t="inlineStr"/>
+      <c r="G143" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H143" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I143" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J143" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 295; Politico-Military Issues: 131; Foreign Economic Policy: 81</t>
@@ -6761,9 +7637,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G144" s="15" t="inlineStr"/>
-      <c r="H144" s="15" t="inlineStr"/>
-      <c r="I144" s="15" t="inlineStr"/>
+      <c r="G144" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H144" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I144" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J144" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 13; Bilateral Relations: 4; Department of State: 3</t>
@@ -6797,9 +7685,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G145" s="15" t="inlineStr"/>
-      <c r="H145" s="15" t="inlineStr"/>
-      <c r="I145" s="15" t="inlineStr"/>
+      <c r="G145" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H145" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I145" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J145" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 317; Politico-Military Issues: 167; Foreign Economic Policy: 104</t>
@@ -6833,9 +7733,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G146" s="15" t="inlineStr"/>
-      <c r="H146" s="15" t="inlineStr"/>
-      <c r="I146" s="15" t="inlineStr"/>
+      <c r="G146" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H146" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I146" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J146" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 22; Foreign Economic Policy: 8; Arms Control and Disarmament: 8</t>
@@ -6869,9 +7781,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G147" s="15" t="inlineStr"/>
-      <c r="H147" s="15" t="inlineStr"/>
-      <c r="I147" s="15" t="inlineStr"/>
+      <c r="G147" s="15" t="inlineStr">
+        <is>
+          <t>Information Programs</t>
+        </is>
+      </c>
+      <c r="H147" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I147" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J147" s="18" t="inlineStr">
         <is>
           <t>Information Programs: 113; Foreign Economic Policy: 79; Politico-Military Issues: 51</t>
@@ -6905,9 +7829,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G148" s="15" t="inlineStr"/>
-      <c r="H148" s="15" t="inlineStr"/>
-      <c r="I148" s="15" t="inlineStr"/>
+      <c r="G148" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H148" s="15" t="inlineStr">
+        <is>
+          <t>Energy and Natural Resources</t>
+        </is>
+      </c>
+      <c r="I148" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J148" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 3; International Law: 2; Global Issues: 2</t>
@@ -6941,9 +7877,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G149" s="15" t="inlineStr"/>
-      <c r="H149" s="15" t="inlineStr"/>
-      <c r="I149" s="15" t="inlineStr"/>
+      <c r="G149" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H149" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I149" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J149" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 11; Foreign Economic Policy: 8; International Law: 5</t>
@@ -6977,9 +7925,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G150" s="15" t="inlineStr"/>
-      <c r="H150" s="15" t="inlineStr"/>
-      <c r="I150" s="15" t="inlineStr"/>
+      <c r="G150" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H150" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I150" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J150" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 2227; Politico-Military Issues: 643; Foreign Economic Policy: 552</t>
@@ -7013,9 +7973,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G151" s="15" t="inlineStr"/>
-      <c r="H151" s="15" t="inlineStr"/>
-      <c r="I151" s="15" t="inlineStr"/>
+      <c r="G151" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H151" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I151" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J151" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 234; Politico-Military Issues: 87; Global Issues: 50</t>
@@ -7049,9 +8021,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G152" s="15" t="inlineStr"/>
-      <c r="H152" s="15" t="inlineStr"/>
-      <c r="I152" s="15" t="inlineStr"/>
+      <c r="G152" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H152" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I152" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J152" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 81; Arms Control and Disarmament: 64; Foreign Economic Policy: 55</t>
@@ -7085,9 +8069,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G153" s="15" t="inlineStr"/>
-      <c r="H153" s="15" t="inlineStr"/>
-      <c r="I153" s="15" t="inlineStr"/>
+      <c r="G153" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H153" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I153" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J153" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 197; Politico-Military Issues: 67; Global Issues: 45</t>
@@ -7121,9 +8117,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G154" s="15" t="inlineStr"/>
-      <c r="H154" s="15" t="inlineStr"/>
-      <c r="I154" s="15" t="inlineStr"/>
+      <c r="G154" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H154" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I154" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J154" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 48; Foreign Economic Policy: 35; Arms Control and Disarmament: 11</t>
@@ -7157,9 +8165,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G155" s="15" t="inlineStr"/>
-      <c r="H155" s="15" t="inlineStr"/>
-      <c r="I155" s="15" t="inlineStr"/>
+      <c r="G155" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H155" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I155" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J155" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 15; Politico-Military Issues: 6; Global Issues: 5</t>
@@ -7193,9 +8213,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G156" s="15" t="inlineStr"/>
-      <c r="H156" s="15" t="inlineStr"/>
-      <c r="I156" s="15" t="inlineStr"/>
+      <c r="G156" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H156" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I156" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J156" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 99; Information Programs: 29; Politico-Military Issues: 27</t>
@@ -7229,9 +8261,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G157" s="15" t="inlineStr"/>
-      <c r="H157" s="15" t="inlineStr"/>
-      <c r="I157" s="15" t="inlineStr"/>
+      <c r="G157" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H157" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I157" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J157" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 552; Politico-Military Issues: 238; International Law: 152</t>
@@ -7265,9 +8309,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G158" s="15" t="inlineStr"/>
-      <c r="H158" s="15" t="inlineStr"/>
-      <c r="I158" s="15" t="inlineStr"/>
+      <c r="G158" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H158" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I158" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J158" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 19; Bilateral Relations: 6; Foreign Economic Policy: 6</t>
@@ -7301,9 +8357,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G159" s="15" t="inlineStr"/>
-      <c r="H159" s="15" t="inlineStr"/>
-      <c r="I159" s="15" t="inlineStr"/>
+      <c r="G159" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H159" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I159" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J159" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 33; Foreign Economic Policy: 11; Global Issues: 9</t>
@@ -7337,9 +8405,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G160" s="15" t="inlineStr"/>
-      <c r="H160" s="15" t="inlineStr"/>
-      <c r="I160" s="15" t="inlineStr"/>
+      <c r="G160" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H160" s="15" t="inlineStr">
+        <is>
+          <t>HIV/AIDS</t>
+        </is>
+      </c>
+      <c r="I160" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J160" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 7; Department of State: 5; Global Issues: 4</t>
@@ -7373,9 +8453,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G161" s="15" t="inlineStr"/>
-      <c r="H161" s="15" t="inlineStr"/>
-      <c r="I161" s="15" t="inlineStr"/>
+      <c r="G161" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H161" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I161" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J161" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 494; Politico-Military Issues: 172; Arms Control and Disarmament: 130</t>
@@ -7409,9 +8501,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G162" s="15" t="inlineStr"/>
-      <c r="H162" s="15" t="inlineStr"/>
-      <c r="I162" s="15" t="inlineStr"/>
+      <c r="G162" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H162" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I162" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J162" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 55; Human Rights: 21; Global Issues: 20</t>
@@ -7445,9 +8549,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G163" s="15" t="inlineStr"/>
-      <c r="H163" s="15" t="inlineStr"/>
-      <c r="I163" s="15" t="inlineStr"/>
+      <c r="G163" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H163" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I163" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J163" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 9; Global Issues: 6; Politico-Military Issues: 2</t>
@@ -7481,9 +8597,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G164" s="15" t="inlineStr"/>
-      <c r="H164" s="15" t="inlineStr"/>
-      <c r="I164" s="15" t="inlineStr"/>
+      <c r="G164" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H164" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I164" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J164" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 98; Politico-Military Issues: 51; Global Issues: 21</t>
@@ -7517,9 +8645,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G165" s="15" t="inlineStr"/>
-      <c r="H165" s="15" t="inlineStr"/>
-      <c r="I165" s="15" t="inlineStr"/>
+      <c r="G165" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H165" s="15" t="inlineStr">
+        <is>
+          <t>Refugees</t>
+        </is>
+      </c>
+      <c r="I165" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J165" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 16; Global Issues: 8; Foreign Economic Policy: 8</t>
@@ -7553,9 +8693,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G166" s="15" t="inlineStr"/>
-      <c r="H166" s="15" t="inlineStr"/>
-      <c r="I166" s="15" t="inlineStr"/>
+      <c r="G166" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H166" s="15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="I166" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J166" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 125; Politico-Military Issues: 42; Human Rights: 33</t>
@@ -7589,9 +8741,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G167" s="15" t="inlineStr"/>
-      <c r="H167" s="15" t="inlineStr"/>
-      <c r="I167" s="15" t="inlineStr"/>
+      <c r="G167" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H167" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I167" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J167" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 373; Politico-Military Issues: 138; Global Issues: 110</t>
@@ -7625,9 +8789,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G168" s="15" t="inlineStr"/>
-      <c r="H168" s="15" t="inlineStr"/>
-      <c r="I168" s="15" t="inlineStr"/>
+      <c r="G168" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H168" s="15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="I168" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J168" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 44; Global Issues: 16; Human Rights: 15</t>
@@ -7661,9 +8837,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G169" s="15" t="inlineStr"/>
-      <c r="H169" s="15" t="inlineStr"/>
-      <c r="I169" s="15" t="inlineStr"/>
+      <c r="G169" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H169" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I169" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J169" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 23; Global Issues: 13; Foreign Economic Policy: 11</t>
@@ -7697,9 +8885,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G170" s="15" t="inlineStr"/>
-      <c r="H170" s="15" t="inlineStr"/>
-      <c r="I170" s="15" t="inlineStr"/>
+      <c r="G170" s="15" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H170" s="15" t="inlineStr">
+        <is>
+          <t>Trade and Commercial Policy/Agreements</t>
+        </is>
+      </c>
+      <c r="I170" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J170" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 31; Global Issues: 11; Information Programs: 9</t>
@@ -7733,9 +8933,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G171" s="15" t="inlineStr"/>
-      <c r="H171" s="15" t="inlineStr"/>
-      <c r="I171" s="15" t="inlineStr"/>
+      <c r="G171" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H171" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I171" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J171" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 28; Global Issues: 15; Politico-Military Issues: 11</t>
@@ -7769,9 +8981,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G172" s="15" t="inlineStr"/>
-      <c r="H172" s="15" t="inlineStr"/>
-      <c r="I172" s="15" t="inlineStr"/>
+      <c r="G172" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H172" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I172" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J172" s="18" t="inlineStr">
         <is>
           <t>Global Issues: 56; Foreign Economic Policy: 55; Human Rights: 23</t>
@@ -7805,9 +9029,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G173" s="15" t="inlineStr"/>
-      <c r="H173" s="15" t="inlineStr"/>
-      <c r="I173" s="15" t="inlineStr"/>
+      <c r="G173" s="15" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H173" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I173" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J173" s="18" t="inlineStr">
         <is>
           <t>Global Issues: 46; Foreign Economic Policy: 34; Politico-Military Issues: 15</t>
@@ -7841,9 +9077,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G174" s="15" t="inlineStr"/>
-      <c r="H174" s="15" t="inlineStr"/>
-      <c r="I174" s="15" t="inlineStr"/>
+      <c r="G174" s="15" t="inlineStr">
+        <is>
+          <t>International Law</t>
+        </is>
+      </c>
+      <c r="H174" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I174" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J174" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 41; Global Issues: 21; Politico-Military Issues: 14</t>
@@ -7877,9 +9125,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G175" s="15" t="inlineStr"/>
-      <c r="H175" s="15" t="inlineStr"/>
-      <c r="I175" s="15" t="inlineStr"/>
+      <c r="G175" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H175" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I175" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J175" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 86; Politico-Military Issues: 68; Foreign Economic Policy: 26</t>
@@ -7913,9 +9173,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G176" s="15" t="inlineStr"/>
-      <c r="H176" s="15" t="inlineStr"/>
-      <c r="I176" s="15" t="inlineStr"/>
+      <c r="G176" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H176" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I176" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J176" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 61; Politico-Military Issues: 31; Global Issues: 27</t>
@@ -7949,9 +9221,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G177" s="15" t="inlineStr"/>
-      <c r="H177" s="15" t="inlineStr"/>
-      <c r="I177" s="15" t="inlineStr"/>
+      <c r="G177" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H177" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I177" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J177" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 340; Politico-Military Issues: 142; Global Issues: 116</t>
@@ -7985,9 +9269,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G178" s="15" t="inlineStr"/>
-      <c r="H178" s="15" t="inlineStr"/>
-      <c r="I178" s="15" t="inlineStr"/>
+      <c r="G178" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H178" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I178" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J178" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 378; Politico-Military Issues: 177; Arms Control and Disarmament: 112</t>
@@ -8021,9 +9317,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G179" s="15" t="inlineStr"/>
-      <c r="H179" s="15" t="inlineStr"/>
-      <c r="I179" s="15" t="inlineStr"/>
+      <c r="G179" s="15" t="inlineStr">
+        <is>
+          <t>International Law</t>
+        </is>
+      </c>
+      <c r="H179" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I179" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J179" s="18" t="inlineStr">
         <is>
           <t>Global Issues: 17; Foreign Economic Policy: 15; International Law: 8</t>
@@ -8057,9 +9365,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G180" s="15" t="inlineStr"/>
-      <c r="H180" s="15" t="inlineStr"/>
-      <c r="I180" s="15" t="inlineStr"/>
+      <c r="G180" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H180" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I180" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J180" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 1293; Politico-Military Issues: 691; Foreign Economic Policy: 541</t>
@@ -8093,9 +9413,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G181" s="15" t="inlineStr"/>
-      <c r="H181" s="15" t="inlineStr"/>
-      <c r="I181" s="15" t="inlineStr"/>
+      <c r="G181" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H181" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I181" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J181" s="18" t="inlineStr">
         <is>
           <t>Human Rights: 7; Global Issues: 5; Bilateral Relations: 3</t>
@@ -8129,9 +9461,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G182" s="15" t="inlineStr"/>
-      <c r="H182" s="15" t="inlineStr"/>
-      <c r="I182" s="15" t="inlineStr"/>
+      <c r="G182" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H182" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I182" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J182" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 30; Global Issues: 16; Politico-Military Issues: 10</t>
@@ -8165,9 +9509,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G183" s="15" t="inlineStr"/>
-      <c r="H183" s="15" t="inlineStr"/>
-      <c r="I183" s="15" t="inlineStr"/>
+      <c r="G183" s="15" t="inlineStr">
+        <is>
+          <t>International Law</t>
+        </is>
+      </c>
+      <c r="H183" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I183" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J183" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 11; Global Issues: 6; Politico-Military Issues: 4</t>
@@ -8201,9 +9557,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G184" s="15" t="inlineStr"/>
-      <c r="H184" s="15" t="inlineStr"/>
-      <c r="I184" s="15" t="inlineStr"/>
+      <c r="G184" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H184" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I184" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J184" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 47; Global Issues: 29; Human Rights: 17</t>
@@ -8237,9 +9605,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G185" s="15" t="inlineStr"/>
-      <c r="H185" s="15" t="inlineStr"/>
-      <c r="I185" s="15" t="inlineStr"/>
+      <c r="G185" s="15" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H185" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I185" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J185" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 36; Politico-Military Issues: 21; Foreign Economic Policy: 19</t>
@@ -8273,9 +9653,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G186" s="15" t="inlineStr"/>
-      <c r="H186" s="15" t="inlineStr"/>
-      <c r="I186" s="15" t="inlineStr"/>
+      <c r="G186" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H186" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I186" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J186" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 14; Foreign Economic Policy: 11; Politico-Military Issues: 4</t>
@@ -8309,9 +9701,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G187" s="15" t="inlineStr"/>
-      <c r="H187" s="15" t="inlineStr"/>
-      <c r="I187" s="15" t="inlineStr"/>
+      <c r="G187" s="15" t="inlineStr">
+        <is>
+          <t>Information Programs</t>
+        </is>
+      </c>
+      <c r="H187" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I187" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J187" s="18" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 52; Politico-Military Issues: 24; Information Programs: 15</t>
@@ -8345,9 +9749,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G188" s="15" t="inlineStr"/>
-      <c r="H188" s="15" t="inlineStr"/>
-      <c r="I188" s="15" t="inlineStr"/>
+      <c r="G188" s="15" t="inlineStr">
+        <is>
+          <t>Science and Technology</t>
+        </is>
+      </c>
+      <c r="H188" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I188" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J188" s="18" t="inlineStr">
         <is>
           <t>Science and Technology: 2; Foreign Economic Policy: 1; Human Rights: 1</t>
@@ -8381,9 +9797,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G189" s="15" t="inlineStr"/>
-      <c r="H189" s="15" t="inlineStr"/>
-      <c r="I189" s="15" t="inlineStr"/>
+      <c r="G189" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H189" s="15" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I189" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J189" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 4; Science and Technology: 3; Foreign Economic Policy: 1</t>
@@ -8417,9 +9845,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G190" s="15" t="inlineStr"/>
-      <c r="H190" s="15" t="inlineStr"/>
-      <c r="I190" s="15" t="inlineStr"/>
+      <c r="G190" s="15" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H190" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I190" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J190" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 7; Politico-Military Issues: 3; Foreign Economic Policy: 3</t>
@@ -8453,9 +9893,21 @@
           <t>keyword + weak co-occurrence</t>
         </is>
       </c>
-      <c r="G191" s="15" t="inlineStr"/>
-      <c r="H191" s="15" t="inlineStr"/>
-      <c r="I191" s="15" t="inlineStr"/>
+      <c r="G191" s="15" t="inlineStr">
+        <is>
+          <t>Warfare</t>
+        </is>
+      </c>
+      <c r="H191" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I191" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J191" s="18" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 3; Arms Control and Disarmament: 2; Bilateral Relations: 2</t>
@@ -8489,9 +9941,21 @@
           <t>co-occurrence (weak)</t>
         </is>
       </c>
-      <c r="G192" s="15" t="inlineStr"/>
-      <c r="H192" s="15" t="inlineStr"/>
-      <c r="I192" s="15" t="inlineStr"/>
+      <c r="G192" s="15" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H192" s="15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I192" s="15" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J192" s="18" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 4; Politico-Military Issues: 4; Bilateral Relations: 1</t>
@@ -8525,9 +9989,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G193" s="19" t="inlineStr"/>
-      <c r="H193" s="19" t="inlineStr"/>
-      <c r="I193" s="19" t="inlineStr"/>
+      <c r="G193" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H193" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I193" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J193" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 18; Foreign Economic Policy: 10; Arms Control and Disarmament: 10</t>
@@ -8561,9 +10037,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G194" s="19" t="inlineStr"/>
-      <c r="H194" s="19" t="inlineStr"/>
-      <c r="I194" s="19" t="inlineStr"/>
+      <c r="G194" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H194" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I194" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J194" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 686; Arms Control and Disarmament: 651; Foreign Economic Policy: 592</t>
@@ -8597,9 +10085,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G195" s="19" t="inlineStr"/>
-      <c r="H195" s="19" t="inlineStr"/>
-      <c r="I195" s="19" t="inlineStr"/>
+      <c r="G195" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H195" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I195" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J195" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 12; International Law: 10; Foreign Economic Policy: 8</t>
@@ -8633,9 +10133,21 @@
           <t>co-occurrence + keyword</t>
         </is>
       </c>
-      <c r="G196" s="19" t="inlineStr"/>
-      <c r="H196" s="19" t="inlineStr"/>
-      <c r="I196" s="19" t="inlineStr"/>
+      <c r="G196" s="19" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H196" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I196" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J196" s="22" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 2026; Politico-Military Issues: 1872; Foreign Economic Policy: 1852</t>
@@ -8669,9 +10181,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G197" s="19" t="inlineStr"/>
-      <c r="H197" s="19" t="inlineStr"/>
-      <c r="I197" s="19" t="inlineStr"/>
+      <c r="G197" s="19" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H197" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I197" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J197" s="22" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 65; Politico-Military Issues: 60; Foreign Economic Policy: 56</t>
@@ -8705,9 +10229,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G198" s="19" t="inlineStr"/>
-      <c r="H198" s="19" t="inlineStr"/>
-      <c r="I198" s="19" t="inlineStr"/>
+      <c r="G198" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H198" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I198" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J198" s="22" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 38; Politico-Military Issues: 22; Global Issues: 22</t>
@@ -8741,9 +10277,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G199" s="19" t="inlineStr"/>
-      <c r="H199" s="19" t="inlineStr"/>
-      <c r="I199" s="19" t="inlineStr"/>
+      <c r="G199" s="19" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H199" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I199" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J199" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 134; Politico-Military Issues: 102; Arms Control and Disarmament: 89</t>
@@ -8777,9 +10325,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G200" s="19" t="inlineStr"/>
-      <c r="H200" s="19" t="inlineStr"/>
-      <c r="I200" s="19" t="inlineStr"/>
+      <c r="G200" s="19" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H200" s="19" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I200" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J200" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 22; Arms Control and Disarmament: 19; Foreign Economic Policy: 17</t>
@@ -8813,9 +10373,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G201" s="19" t="inlineStr"/>
-      <c r="H201" s="19" t="inlineStr"/>
-      <c r="I201" s="19" t="inlineStr"/>
+      <c r="G201" s="19" t="inlineStr">
+        <is>
+          <t>Science and Technology</t>
+        </is>
+      </c>
+      <c r="H201" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I201" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J201" s="22" t="inlineStr">
         <is>
           <t>Information Programs: 10; Arms Control and Disarmament: 8; Science and Technology: 7</t>
@@ -8849,9 +10421,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G202" s="19" t="inlineStr"/>
-      <c r="H202" s="19" t="inlineStr"/>
-      <c r="I202" s="19" t="inlineStr"/>
+      <c r="G202" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H202" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I202" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J202" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 276; Arms Control and Disarmament: 173; Politico-Military Issues: 160</t>
@@ -8885,9 +10469,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G203" s="19" t="inlineStr"/>
-      <c r="H203" s="19" t="inlineStr"/>
-      <c r="I203" s="19" t="inlineStr"/>
+      <c r="G203" s="19" t="inlineStr">
+        <is>
+          <t>Human Rights</t>
+        </is>
+      </c>
+      <c r="H203" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I203" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J203" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 10; Politico-Military Issues: 10; Information Programs: 6</t>
@@ -8921,9 +10517,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G204" s="19" t="inlineStr"/>
-      <c r="H204" s="19" t="inlineStr"/>
-      <c r="I204" s="19" t="inlineStr"/>
+      <c r="G204" s="19" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H204" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I204" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J204" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 5; Warfare: 4; Foreign Economic Policy: 3</t>
@@ -8957,9 +10565,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G205" s="19" t="inlineStr"/>
-      <c r="H205" s="19" t="inlineStr"/>
-      <c r="I205" s="19" t="inlineStr"/>
+      <c r="G205" s="19" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H205" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I205" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J205" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 972; Politico-Military Issues: 654; Arms Control and Disarmament: 421</t>
@@ -8993,9 +10613,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G206" s="19" t="inlineStr"/>
-      <c r="H206" s="19" t="inlineStr"/>
-      <c r="I206" s="19" t="inlineStr"/>
+      <c r="G206" s="19" t="inlineStr">
+        <is>
+          <t>Information Programs</t>
+        </is>
+      </c>
+      <c r="H206" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I206" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J206" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 9; Bilateral Relations: 7; Information Programs: 5</t>
@@ -9029,9 +10661,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G207" s="19" t="inlineStr"/>
-      <c r="H207" s="19" t="inlineStr"/>
-      <c r="I207" s="19" t="inlineStr"/>
+      <c r="G207" s="19" t="inlineStr">
+        <is>
+          <t>Global Issues</t>
+        </is>
+      </c>
+      <c r="H207" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I207" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J207" s="22" t="inlineStr">
         <is>
           <t>Arms Control and Disarmament: 18; Foreign Economic Policy: 9; Science and Technology: 7</t>
@@ -9065,9 +10709,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G208" s="19" t="inlineStr"/>
-      <c r="H208" s="19" t="inlineStr"/>
-      <c r="I208" s="19" t="inlineStr"/>
+      <c r="G208" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H208" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I208" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J208" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 19; Arms Control and Disarmament: 11; Politico-Military Issues: 9</t>
@@ -9101,9 +10757,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G209" s="19" t="inlineStr"/>
-      <c r="H209" s="19" t="inlineStr"/>
-      <c r="I209" s="19" t="inlineStr"/>
+      <c r="G209" s="19" t="inlineStr">
+        <is>
+          <t>Information Programs</t>
+        </is>
+      </c>
+      <c r="H209" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I209" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J209" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 4; Information Programs: 3; Science and Technology: 3</t>
@@ -9137,9 +10805,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G210" s="19" t="inlineStr"/>
-      <c r="H210" s="19" t="inlineStr"/>
-      <c r="I210" s="19" t="inlineStr"/>
+      <c r="G210" s="19" t="inlineStr">
+        <is>
+          <t>Information Programs</t>
+        </is>
+      </c>
+      <c r="H210" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I210" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J210" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 166; Politico-Military Issues: 114; Arms Control and Disarmament: 76</t>
@@ -9173,9 +10853,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G211" s="19" t="inlineStr"/>
-      <c r="H211" s="19" t="inlineStr"/>
-      <c r="I211" s="19" t="inlineStr"/>
+      <c r="G211" s="19" t="inlineStr">
+        <is>
+          <t>Politico-Military Issues</t>
+        </is>
+      </c>
+      <c r="H211" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I211" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J211" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 5; Politico-Military Issues: 4; Bilateral Relations: 2</t>
@@ -9209,9 +10901,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G212" s="19" t="inlineStr"/>
-      <c r="H212" s="19" t="inlineStr"/>
-      <c r="I212" s="19" t="inlineStr"/>
+      <c r="G212" s="19" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H212" s="19" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I212" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J212" s="22" t="inlineStr">
         <is>
           <t>Foreign Economic Policy: 11; Politico-Military Issues: 9; Information Programs: 5</t>
@@ -9245,9 +10949,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G213" s="19" t="inlineStr"/>
-      <c r="H213" s="19" t="inlineStr"/>
-      <c r="I213" s="19" t="inlineStr"/>
+      <c r="G213" s="19" t="inlineStr">
+        <is>
+          <t>Foreign Economic Policy</t>
+        </is>
+      </c>
+      <c r="H213" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I213" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J213" s="22" t="inlineStr">
         <is>
           <t>Information Programs: 5; Global Issues: 4; Arms Control and Disarmament: 4</t>
@@ -9281,9 +10997,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G214" s="19" t="inlineStr"/>
-      <c r="H214" s="19" t="inlineStr"/>
-      <c r="I214" s="19" t="inlineStr"/>
+      <c r="G214" s="19" t="inlineStr">
+        <is>
+          <t>Arms Control and Disarmament</t>
+        </is>
+      </c>
+      <c r="H214" s="19" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons</t>
+        </is>
+      </c>
+      <c r="I214" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J214" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 112; Foreign Economic Policy: 111; Arms Control and Disarmament: 58</t>
@@ -9317,9 +11045,21 @@
           <t>keyword only</t>
         </is>
       </c>
-      <c r="G215" s="19" t="inlineStr"/>
-      <c r="H215" s="19" t="inlineStr"/>
-      <c r="I215" s="19" t="inlineStr"/>
+      <c r="G215" s="19" t="inlineStr">
+        <is>
+          <t>International Law</t>
+        </is>
+      </c>
+      <c r="H215" s="19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I215" s="19" t="inlineStr">
+        <is>
+          <t>accept</t>
+        </is>
+      </c>
       <c r="J215" s="22" t="inlineStr">
         <is>
           <t>Politico-Military Issues: 34; Foreign Economic Policy: 24; Information Programs: 15</t>

</xml_diff>